<commit_message>
Partial completion of partial system
</commit_message>
<xml_diff>
--- a/Concrete_Requisition_Slip.xlsx
+++ b/Concrete_Requisition_Slip.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Michael\L_T internship\concrete_recon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F96755-D5A5-4839-9D78-8F63F257B4D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BDB5645-562A-4057-996D-C4FCAD16D67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E0C9EC41-F8DE-4671-8732-902ABF7DE422}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19926" uniqueCount="1258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19927" uniqueCount="1258">
   <si>
     <t>Location</t>
   </si>
@@ -5839,7 +5837,9 @@
       <c r="E93" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F93" s="5"/>
+      <c r="F93" s="5" t="s">
+        <v>610</v>
+      </c>
     </row>
     <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3" t="s">

</xml_diff>